<commit_message>
chore: sync verified final paper analysis files
</commit_message>
<xml_diff>
--- a/results/final/Germany_Results_v3.xlsx
+++ b/results/final/Germany_Results_v3.xlsx
@@ -1,49 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dezernatzukunft.sharepoint.com/sites/DZ-Schalte/Freigegebene Dokumente/2_Projekte/Fiskalpolitik/F48_EUCAM_DSA_Reformvorschlag/03_Modell/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_5D8791B8B8D97DB2FEB36C2B99A3845721D77983" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09B552A8-494B-4F1E-80FC-5CB726D48BCE}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="IQ_CH">110000</definedName>
-    <definedName name="IQ_CQ">5000</definedName>
-    <definedName name="IQ_CY">10000</definedName>
-    <definedName name="IQ_DAILY">500000</definedName>
-    <definedName name="IQ_FH">100000</definedName>
-    <definedName name="IQ_FQ">500</definedName>
-    <definedName name="IQ_FWD_CY" hidden="1">10001</definedName>
-    <definedName name="IQ_FWD_CY1" hidden="1">10002</definedName>
-    <definedName name="IQ_FWD_CY2" hidden="1">10003</definedName>
-    <definedName name="IQ_FWD_FY" hidden="1">1001</definedName>
-    <definedName name="IQ_FWD_FY1" hidden="1">1002</definedName>
-    <definedName name="IQ_FWD_FY2" hidden="1">1003</definedName>
-    <definedName name="IQ_FWD_Q" hidden="1">501</definedName>
-    <definedName name="IQ_FWD_Q1" hidden="1">502</definedName>
-    <definedName name="IQ_FWD_Q2" hidden="1">503</definedName>
-    <definedName name="IQ_FY">1000</definedName>
-    <definedName name="IQ_LATESTK" hidden="1">1000</definedName>
-    <definedName name="IQ_LATESTQ" hidden="1">500</definedName>
-    <definedName name="IQ_LTM">2000</definedName>
-    <definedName name="IQ_LTMMONTH" hidden="1">120000</definedName>
-    <definedName name="IQ_MONTH">15000</definedName>
-    <definedName name="IQ_NTM">6000</definedName>
-    <definedName name="IQ_TODAY" hidden="1">0</definedName>
-    <definedName name="IQ_WEEK">50000</definedName>
-    <definedName name="IQ_YTD">3000</definedName>
-    <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
-  </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -92,8 +58,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -152,25 +118,17 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -208,7 +166,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -242,7 +200,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -277,10 +234,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -453,11 +409,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -498,7 +454,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -533,7 +489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -544,13 +500,13 @@
         <v>-1.3</v>
       </c>
       <c r="D3">
-        <v>-57770886295.416542</v>
+        <v>-57770886295.41654</v>
       </c>
       <c r="E3">
-        <v>-57771328564.810158</v>
+        <v>-57771328564.81016</v>
       </c>
       <c r="F3">
-        <v>63.903263408415107</v>
+        <v>63.90326340841511</v>
       </c>
       <c r="G3">
         <v>64.02625198677093</v>
@@ -565,16 +521,16 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>-442269.39361572271</v>
+        <v>-442269.3936157227</v>
       </c>
       <c r="L3">
         <v>0.122988578355816</v>
       </c>
       <c r="M3">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -585,16 +541,16 @@
         <v>-1.8</v>
       </c>
       <c r="D4">
-        <v>-83616775794.921982</v>
+        <v>-83616775794.92198</v>
       </c>
       <c r="E4">
-        <v>-83898251818.116333</v>
+        <v>-83898251818.11633</v>
       </c>
       <c r="F4">
-        <v>64.547314765242163</v>
+        <v>64.54731476524216</v>
       </c>
       <c r="G4">
-        <v>64.540308533630352</v>
+        <v>64.54030853363035</v>
       </c>
       <c r="H4">
         <v>0.9</v>
@@ -609,13 +565,13 @@
         <v>-281476023.1943512</v>
       </c>
       <c r="L4">
-        <v>-7.0062316118111312E-3</v>
+        <v>-0.007006231611811131</v>
       </c>
       <c r="M4">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -626,16 +582,16 @@
         <v>-1.272077026367187</v>
       </c>
       <c r="D5">
-        <v>-59612604834.773399</v>
+        <v>-59612604834.7734</v>
       </c>
       <c r="E5">
-        <v>-61486544300.176781</v>
+        <v>-61486544300.17678</v>
       </c>
       <c r="F5">
-        <v>65.387152160561484</v>
+        <v>65.38715216056148</v>
       </c>
       <c r="G5">
-        <v>65.246122024599629</v>
+        <v>65.24612202459963</v>
       </c>
       <c r="H5">
         <v>0.9</v>
@@ -644,60 +600,60 @@
         <v>1.152974677827046</v>
       </c>
       <c r="J5">
-        <v>-3.0548095703125E-2</v>
+        <v>-0.030548095703125</v>
       </c>
       <c r="K5">
-        <v>-1873939465.4033811</v>
+        <v>-1873939465.403381</v>
       </c>
       <c r="L5">
-        <v>-0.14103013596185579</v>
+        <v>-0.1410301359618558</v>
       </c>
       <c r="M5">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6">
         <v>2028</v>
       </c>
       <c r="B6">
-        <v>-0.68305786132812496</v>
+        <v>-0.683057861328125</v>
       </c>
       <c r="C6">
-        <v>-0.74415405273437496</v>
+        <v>-0.744154052734375</v>
       </c>
       <c r="D6">
-        <v>-33917557048.615822</v>
+        <v>-33917557048.61582</v>
       </c>
       <c r="E6">
-        <v>-37310313568.569771</v>
+        <v>-37310313568.56977</v>
       </c>
       <c r="F6">
-        <v>65.762353056507905</v>
+        <v>65.76235305650791</v>
       </c>
       <c r="G6">
-        <v>65.508227637451256</v>
+        <v>65.50822763745126</v>
       </c>
       <c r="H6">
         <v>0.9</v>
       </c>
       <c r="I6">
-        <v>1.1529746778270229</v>
+        <v>1.152974677827023</v>
       </c>
       <c r="J6">
-        <v>-6.109619140625E-2</v>
+        <v>-0.06109619140625</v>
       </c>
       <c r="K6">
-        <v>-3392756519.9539528</v>
+        <v>-3392756519.953953</v>
       </c>
       <c r="L6">
-        <v>-0.25412541905664909</v>
+        <v>-0.2541254190566491</v>
       </c>
       <c r="M6">
-        <v>0.25297467782702332</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270233</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -708,16 +664,16 @@
         <v>-0.2162310791015625</v>
       </c>
       <c r="D7">
-        <v>-6393696759.3500481</v>
+        <v>-6393696759.350048</v>
       </c>
       <c r="E7">
-        <v>-11236615580.690889</v>
+        <v>-11236615580.69089</v>
       </c>
       <c r="F7">
-        <v>65.729006655684103</v>
+        <v>65.7290066556841</v>
       </c>
       <c r="G7">
-        <v>65.386462366569006</v>
+        <v>65.38646236656901</v>
       </c>
       <c r="H7">
         <v>0.9</v>
@@ -726,39 +682,39 @@
         <v>1.152974677827046</v>
       </c>
       <c r="J7">
-        <v>-9.1644287109375E-2</v>
+        <v>-0.091644287109375</v>
       </c>
       <c r="K7">
-        <v>-4842918821.3408394</v>
+        <v>-4842918821.340839</v>
       </c>
       <c r="L7">
-        <v>-0.34254428911509649</v>
+        <v>-0.3425442891150965</v>
       </c>
       <c r="M7">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8">
         <v>2030</v>
       </c>
       <c r="B8">
-        <v>0.43388427734375001</v>
+        <v>0.43388427734375</v>
       </c>
       <c r="C8">
-        <v>0.31169189453125001</v>
+        <v>0.31169189453125</v>
       </c>
       <c r="D8">
-        <v>23017994340.230659</v>
+        <v>23017994340.23066</v>
       </c>
       <c r="E8">
-        <v>16789765683.572809</v>
+        <v>16789765683.57281</v>
       </c>
       <c r="F8">
-        <v>65.218196430297567</v>
+        <v>65.21819643029757</v>
       </c>
       <c r="G8">
-        <v>64.814965636015373</v>
+        <v>64.81496563601537</v>
       </c>
       <c r="H8">
         <v>0.9</v>
@@ -770,16 +726,16 @@
         <v>-0.1221923828125</v>
       </c>
       <c r="K8">
-        <v>-6228228656.6578522</v>
+        <v>-6228228656.657852</v>
       </c>
       <c r="L8">
-        <v>-0.40323079428219438</v>
+        <v>-0.4032307942821944</v>
       </c>
       <c r="M8">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -790,10 +746,10 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D9">
-        <v>54377284956.391296</v>
+        <v>54377284956.3913</v>
       </c>
       <c r="E9">
-        <v>46839326958.697777</v>
+        <v>46839326958.69778</v>
       </c>
       <c r="F9">
         <v>64.28913795606725</v>
@@ -811,16 +767,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K9">
-        <v>-7537957997.6935272</v>
+        <v>-7537957997.693527</v>
       </c>
       <c r="L9">
-        <v>-0.43458688093132031</v>
+        <v>-0.4345868809313203</v>
       </c>
       <c r="M9">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -831,16 +787,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D10">
-        <v>56410062696.785698</v>
+        <v>56410062696.7857</v>
       </c>
       <c r="E10">
         <v>48705817347.65554</v>
       </c>
       <c r="F10">
-        <v>63.085297332407272</v>
+        <v>63.08529733240727</v>
       </c>
       <c r="G10">
-        <v>62.648943154679117</v>
+        <v>62.64894315467912</v>
       </c>
       <c r="H10">
         <v>0.9</v>
@@ -852,16 +808,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K10">
-        <v>-7704245349.1301575</v>
+        <v>-7704245349.130157</v>
       </c>
       <c r="L10">
-        <v>-0.43635417772814827</v>
+        <v>-0.4363541777281483</v>
       </c>
       <c r="M10">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -872,16 +828,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D11">
-        <v>58460740950.770599</v>
+        <v>58460740950.7706</v>
       </c>
       <c r="E11">
-        <v>50596460835.952972</v>
+        <v>50596460835.95297</v>
       </c>
       <c r="F11">
-        <v>61.921429198619123</v>
+        <v>61.92142919861912</v>
       </c>
       <c r="G11">
-        <v>61.491792839911177</v>
+        <v>61.49179283991118</v>
       </c>
       <c r="H11">
         <v>0.9</v>
@@ -896,13 +852,13 @@
         <v>-7864280114.817627</v>
       </c>
       <c r="L11">
-        <v>-0.42963635870793843</v>
+        <v>-0.4296363587079384</v>
       </c>
       <c r="M11">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -913,16 +869,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D12">
-        <v>60584997951.980766</v>
+        <v>60584997951.98077</v>
       </c>
       <c r="E12">
-        <v>52559706432.911324</v>
+        <v>52559706432.91132</v>
       </c>
       <c r="F12">
-        <v>60.722935134709559</v>
+        <v>60.72293513470956</v>
       </c>
       <c r="G12">
-        <v>60.308844987945982</v>
+        <v>60.30884498794598</v>
       </c>
       <c r="H12">
         <v>0.9</v>
@@ -934,16 +890,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K12">
-        <v>-8025291519.0694504</v>
+        <v>-8025291519.06945</v>
       </c>
       <c r="L12">
-        <v>-0.41409014676357708</v>
+        <v>-0.4140901467635771</v>
       </c>
       <c r="M12">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -957,13 +913,13 @@
         <v>62475128718.08667</v>
       </c>
       <c r="E13">
-        <v>54335352082.677116</v>
+        <v>54335352082.67712</v>
       </c>
       <c r="F13">
-        <v>59.950218914792941</v>
+        <v>59.95021891479294</v>
       </c>
       <c r="G13">
-        <v>59.543691148133981</v>
+        <v>59.54369114813398</v>
       </c>
       <c r="H13">
         <v>0.9</v>
@@ -975,16 +931,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K13">
-        <v>-8139776635.4095459</v>
+        <v>-8139776635.409546</v>
       </c>
       <c r="L13">
-        <v>-0.40652776665896079</v>
+        <v>-0.4065277666589608</v>
       </c>
       <c r="M13">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -995,16 +951,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D14">
-        <v>64424227783.833527</v>
+        <v>64424227783.83353</v>
       </c>
       <c r="E14">
-        <v>56170985081.831131</v>
+        <v>56170985081.83113</v>
       </c>
       <c r="F14">
-        <v>59.256771236652099</v>
+        <v>59.2567712366521</v>
       </c>
       <c r="G14">
-        <v>58.859403346784113</v>
+        <v>58.85940334678411</v>
       </c>
       <c r="H14">
         <v>0.9</v>
@@ -1016,16 +972,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K14">
-        <v>-8253242702.0023956</v>
+        <v>-8253242702.002396</v>
       </c>
       <c r="L14">
-        <v>-0.39736788986799348</v>
+        <v>-0.3973678898679935</v>
       </c>
       <c r="M14">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -1036,13 +992,13 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D15">
-        <v>66434134842.233543</v>
+        <v>66434134842.23354</v>
       </c>
       <c r="E15">
-        <v>58068632007.065079</v>
+        <v>58068632007.06508</v>
       </c>
       <c r="F15">
-        <v>58.624861585666309</v>
+        <v>58.62486158566631</v>
       </c>
       <c r="G15">
         <v>58.23800883565346</v>
@@ -1057,16 +1013,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K15">
-        <v>-8365502835.1684647</v>
+        <v>-8365502835.168465</v>
       </c>
       <c r="L15">
-        <v>-0.38685275001284941</v>
+        <v>-0.3868527500128494</v>
       </c>
       <c r="M15">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -1077,16 +1033,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D16">
-        <v>68506746981.041542</v>
+        <v>68506746981.04154</v>
       </c>
       <c r="E16">
-        <v>60030387899.724182</v>
+        <v>60030387899.72418</v>
       </c>
       <c r="F16">
-        <v>58.026181834438432</v>
+        <v>58.02618183443843</v>
       </c>
       <c r="G16">
-        <v>57.651021209793562</v>
+        <v>57.65102120979356</v>
       </c>
       <c r="H16">
         <v>0.9</v>
@@ -1098,16 +1054,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K16">
-        <v>-8476359081.3173599</v>
+        <v>-8476359081.31736</v>
       </c>
       <c r="L16">
-        <v>-0.37516062464487021</v>
+        <v>-0.3751606246448702</v>
       </c>
       <c r="M16">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -1118,16 +1074,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D17">
-        <v>70644020473.356079</v>
+        <v>70644020473.35608</v>
       </c>
       <c r="E17">
-        <v>62058418578.775963</v>
+        <v>62058418578.77596</v>
       </c>
       <c r="F17">
-        <v>57.448236955429223</v>
+        <v>57.44823695542922</v>
       </c>
       <c r="G17">
-        <v>57.085853006404882</v>
+        <v>57.08585300640488</v>
       </c>
       <c r="H17">
         <v>0.9</v>
@@ -1139,16 +1095,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K17">
-        <v>-8585601894.5801239</v>
+        <v>-8585601894.580124</v>
       </c>
       <c r="L17">
-        <v>-0.36238394902434118</v>
+        <v>-0.3623839490243412</v>
       </c>
       <c r="M17">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -1159,16 +1115,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D18">
-        <v>72847972624.083832</v>
+        <v>72847972624.08383</v>
       </c>
       <c r="E18">
-        <v>64154963031.919037</v>
+        <v>64154963031.91904</v>
       </c>
       <c r="F18">
-        <v>56.880805191428188</v>
+        <v>56.88080519142819</v>
       </c>
       <c r="G18">
-        <v>56.532232568156857</v>
+        <v>56.53223256815686</v>
       </c>
       <c r="H18">
         <v>0.9</v>
@@ -1180,16 +1136,16 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K18">
-        <v>-8693009592.1647949</v>
+        <v>-8693009592.164795</v>
       </c>
       <c r="L18">
-        <v>-0.34857262327133748</v>
+        <v>-0.3485726232713375</v>
       </c>
       <c r="M18">
-        <v>0.25297467782704552</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0.2529746778270455</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -1200,16 +1156,16 @@
         <v>0.8396148681640625</v>
       </c>
       <c r="D19">
-        <v>75120683674.009979</v>
+        <v>75120683674.00998</v>
       </c>
       <c r="E19">
-        <v>66322335887.471764</v>
+        <v>66322335887.47176</v>
       </c>
       <c r="F19">
-        <v>56.329544747893692</v>
+        <v>56.32954474789369</v>
       </c>
       <c r="G19">
-        <v>55.995802171946082</v>
+        <v>55.99580217194608</v>
       </c>
       <c r="H19">
         <v>0.9</v>
@@ -1221,13 +1177,13 @@
         <v>-0.152740478515625</v>
       </c>
       <c r="K19">
-        <v>-8798347786.5382156</v>
+        <v>-8798347786.538216</v>
       </c>
       <c r="L19">
-        <v>-0.33374257594760343</v>
+        <v>-0.3337425759476034</v>
       </c>
       <c r="M19">
-        <v>0.25297467782704552</v>
+        <v>0.2529746778270455</v>
       </c>
     </row>
   </sheetData>
@@ -1236,28 +1192,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f58ec337-e214-4ba4-98b7-7d376ec9c384">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="bce3f25c-6c94-415f-946f-6384d96b8749" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100CBE255276945314790992D07276A2E9C" ma:contentTypeVersion="18" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="8675bac851cd0906af82d9b344b788d4">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f58ec337-e214-4ba4-98b7-7d376ec9c384" xmlns:ns3="bce3f25c-6c94-415f-946f-6384d96b8749" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0e9d441ae2c0b8244772fe863691a22" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100CBE255276945314790992D07276A2E9C" ma:contentTypeVersion="18" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e852c1eda4579854110eaa5540fcc087">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f58ec337-e214-4ba4-98b7-7d376ec9c384" xmlns:ns3="bce3f25c-6c94-415f-946f-6384d96b8749" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fcb9988e94d3ed424c91cebd889f8959" ns2:_="" ns3:_="">
     <xsd:import namespace="f58ec337-e214-4ba4-98b7-7d376ec9c384"/>
     <xsd:import namespace="bce3f25c-6c94-415f-946f-6384d96b8749"/>
     <xsd:element name="properties">
@@ -1510,25 +1446,34 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f58ec337-e214-4ba4-98b7-7d376ec9c384">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="bce3f25c-6c94-415f-946f-6384d96b8749" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C5F05C0-99B4-4702-9339-C4AA49D3CB54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f58ec337-e214-4ba4-98b7-7d376ec9c384"/>
-    <ds:schemaRef ds:uri="bce3f25c-6c94-415f-946f-6384d96b8749"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{389C3A63-FC26-4A69-BE59-52A531BE3BCB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38C005E5-36FE-4A6D-B83C-70CC347D1EAD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38C005E5-36FE-4A6D-B83C-70CC347D1EAD}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4955C650-203E-4AEC-93B0-DAF985687FB6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C5F05C0-99B4-4702-9339-C4AA49D3CB54}"/>
 </file>
</xml_diff>